<commit_message>
Customer Churn Project Documentation
Added the Excel documentation file containing project details, analysis information, and supporting documentation for the Customer Churn Prediction project.
</commit_message>
<xml_diff>
--- a/README.xlsx
+++ b/README.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ff802e6ab1614350/Desktop/ML Project P1 and P2 - Airbnb Price Prediction ^M Churn Prediction/Airbnb Price Prediction and Insights/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ff802e6ab1614350/Desktop/ML Project P1 and P2 - Airbnb Price Prediction ^M Churn Prediction/Customer Churn Prediction/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="11_F25DC773A252ABDACC10483C295D6BEC5BDE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E371AB3B-39A3-44FE-A236-CF6CB4E1D9D3}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="11_F25DC773A252ABDACC10483C295D6BEC5BDE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FBEF5DDF-E6DC-4B3E-84F1-63CDDBC8675B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
     <t>Video Link :-</t>
   </si>
   <si>
-    <t>Click  Here</t>
+    <t>Click Here</t>
   </si>
 </sst>
 </file>
@@ -46,17 +46,17 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
+      <b/>
       <sz val="11"/>
-      <color theme="10"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <u/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -81,12 +81,12 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -103,10 +103,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -372,25 +368,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="H16:I16"/>
+  <dimension ref="I13:J13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="8" max="8" width="12.88671875" customWidth="1"/>
-    <col min="9" max="9" width="14.88671875" customWidth="1"/>
+    <col min="9" max="9" width="13.5546875" customWidth="1"/>
+    <col min="10" max="10" width="10.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="16" spans="8:9" x14ac:dyDescent="0.3">
-      <c r="H16" s="2" t="s">
+    <row r="13" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I13" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="I16" s="1" t="s">
+      <c r="J13" s="1" t="s">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="I16" r:id="rId1" xr:uid="{48574BE3-D12B-4F6E-BD65-04B18FEF689F}"/>
+    <hyperlink ref="J13" r:id="rId1" xr:uid="{4803ED68-5719-43FA-80BA-5948ABA19E5D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>